<commit_message>
Refactor Azure Entra Offboarding Report script: removed the script file, updated guest invite message in Graph-GuestInvitesPersonal, enhanced group creation in Graph-New-UnifiedGroup, modified connection parameters in Module-Connect, added new application access policy in Test.ps1, and implemented email sending functionality in test123.ps1.
</commit_message>
<xml_diff>
--- a/Input Data/ContractorList.xlsx
+++ b/Input Data/ContractorList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49754D9-4447-4970-A4BB-DF32858FC04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F937D7D4-8FD2-4543-8F08-5620F7FF7484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E27B5980-8A07-4A5D-9AD2-51AB851DDA69}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E27B5980-8A07-4A5D-9AD2-51AB851DDA69}"/>
   </bookViews>
   <sheets>
     <sheet name="EntraID" sheetId="1" r:id="rId1"/>
@@ -162,9 +162,6 @@
     <t>ENC-WALL</t>
   </si>
   <si>
-    <t>ENC-TAIL</t>
-  </si>
-  <si>
     <t>ENGINE</t>
   </si>
   <si>
@@ -202,6 +199,9 @@
   </si>
   <si>
     <t>svcaccount</t>
+  </si>
+  <si>
+    <t>ENC-HAIL</t>
   </si>
 </sst>
 </file>
@@ -629,7 +629,7 @@
         <v>32</v>
       </c>
       <c r="N1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -659,13 +659,13 @@
         <v>46258</v>
       </c>
       <c r="H2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" t="s">
         <v>48</v>
       </c>
-      <c r="I2" t="s">
-        <v>49</v>
-      </c>
       <c r="J2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K2" t="s">
         <v>7</v>
@@ -677,7 +677,7 @@
         <v>33</v>
       </c>
       <c r="N2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -707,13 +707,13 @@
         <v>46258</v>
       </c>
       <c r="H3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" t="s">
         <v>48</v>
       </c>
-      <c r="I3" t="s">
-        <v>49</v>
-      </c>
       <c r="J3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K3" t="s">
         <v>7</v>
@@ -722,10 +722,10 @@
         <v>18</v>
       </c>
       <c r="M3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -755,13 +755,13 @@
         <v>46258</v>
       </c>
       <c r="H4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" t="s">
         <v>48</v>
       </c>
-      <c r="I4" t="s">
-        <v>49</v>
-      </c>
       <c r="J4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K4" t="s">
         <v>7</v>
@@ -770,10 +770,10 @@
         <v>12</v>
       </c>
       <c r="M4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -803,13 +803,13 @@
         <v>46258</v>
       </c>
       <c r="H5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" t="s">
         <v>48</v>
       </c>
-      <c r="I5" t="s">
-        <v>49</v>
-      </c>
       <c r="J5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K5" t="s">
         <v>7</v>
@@ -818,10 +818,10 @@
         <v>13</v>
       </c>
       <c r="M5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -851,13 +851,13 @@
         <v>46258</v>
       </c>
       <c r="H6" t="s">
+        <v>47</v>
+      </c>
+      <c r="I6" t="s">
         <v>48</v>
       </c>
-      <c r="I6" t="s">
-        <v>49</v>
-      </c>
       <c r="J6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K6" t="s">
         <v>7</v>
@@ -866,10 +866,10 @@
         <v>24</v>
       </c>
       <c r="M6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -899,13 +899,13 @@
         <v>46258</v>
       </c>
       <c r="H7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" t="s">
         <v>48</v>
       </c>
-      <c r="I7" t="s">
-        <v>49</v>
-      </c>
       <c r="J7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K7" t="s">
         <v>7</v>
@@ -914,23 +914,23 @@
         <v>17</v>
       </c>
       <c r="M7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
-        <v>ENC-TAIL@erock.com</v>
+        <v>ENC-HAIL@erock.com</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="1"/>
-        <v>ENC-TAIL</v>
+        <v>ENC-HAIL</v>
       </c>
       <c r="D8" t="e">
         <f t="shared" si="3"/>
@@ -947,13 +947,13 @@
         <v>46258</v>
       </c>
       <c r="H8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" t="s">
         <v>48</v>
       </c>
-      <c r="I8" t="s">
-        <v>49</v>
-      </c>
       <c r="J8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K8" t="s">
         <v>7</v>
@@ -962,15 +962,15 @@
         <v>16</v>
       </c>
       <c r="M8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -995,13 +995,13 @@
         <v>46258</v>
       </c>
       <c r="H9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" t="s">
         <v>48</v>
       </c>
-      <c r="I9" t="s">
-        <v>49</v>
-      </c>
       <c r="J9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K9" t="s">
         <v>7</v>
@@ -1010,15 +1010,15 @@
         <v>15</v>
       </c>
       <c r="M9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -1043,13 +1043,13 @@
         <v>46258</v>
       </c>
       <c r="H10" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10" t="s">
         <v>48</v>
       </c>
-      <c r="I10" t="s">
-        <v>49</v>
-      </c>
       <c r="J10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K10" t="s">
         <v>7</v>
@@ -1058,15 +1058,15 @@
         <v>14</v>
       </c>
       <c r="M10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -1091,13 +1091,13 @@
         <v>46258</v>
       </c>
       <c r="H11" t="s">
+        <v>47</v>
+      </c>
+      <c r="I11" t="s">
         <v>48</v>
       </c>
-      <c r="I11" t="s">
-        <v>49</v>
-      </c>
       <c r="J11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K11" t="s">
         <v>7</v>
@@ -1106,15 +1106,15 @@
         <v>19</v>
       </c>
       <c r="M11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
@@ -1139,13 +1139,13 @@
         <v>46258</v>
       </c>
       <c r="H12" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" t="s">
         <v>48</v>
       </c>
-      <c r="I12" t="s">
-        <v>49</v>
-      </c>
       <c r="J12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K12" t="s">
         <v>7</v>
@@ -1154,15 +1154,15 @@
         <v>20</v>
       </c>
       <c r="M12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -1187,13 +1187,13 @@
         <v>46258</v>
       </c>
       <c r="H13" t="s">
+        <v>47</v>
+      </c>
+      <c r="I13" t="s">
         <v>48</v>
       </c>
-      <c r="I13" t="s">
-        <v>49</v>
-      </c>
       <c r="J13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K13" t="s">
         <v>7</v>
@@ -1202,15 +1202,15 @@
         <v>21</v>
       </c>
       <c r="M13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
@@ -1235,13 +1235,13 @@
         <v>46258</v>
       </c>
       <c r="H14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I14" t="s">
         <v>48</v>
       </c>
-      <c r="I14" t="s">
-        <v>49</v>
-      </c>
       <c r="J14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K14" t="s">
         <v>7</v>
@@ -1250,15 +1250,15 @@
         <v>22</v>
       </c>
       <c r="M14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -1283,13 +1283,13 @@
         <v>46258</v>
       </c>
       <c r="H15" t="s">
+        <v>47</v>
+      </c>
+      <c r="I15" t="s">
         <v>48</v>
       </c>
-      <c r="I15" t="s">
-        <v>49</v>
-      </c>
       <c r="J15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K15" t="s">
         <v>7</v>
@@ -1298,10 +1298,10 @@
         <v>23</v>
       </c>
       <c r="M15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>